<commit_message>
Correct HRM-Text exact benchmark scoring
</commit_message>
<xml_diff>
--- a/outputs/qwen_hrm_metrics/qwen_hrm_conversion_metrics.xlsx
+++ b/outputs/qwen_hrm_metrics/qwen_hrm_conversion_metrics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R489b153ed78248b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Runs" sheetId="2" r:id="R5fff4c1c869645d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Outcomes" sheetId="3" r:id="R5a78dbad18044a85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sweep Runs" sheetId="4" r:id="Rba35bacd1ac04cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Runs" sheetId="5" r:id="Ref627b9935584f11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Outcomes" sheetId="6" r:id="R8974cf3ece8046ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" r:id="R258aeff5b1f94c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9f695a055fe4498d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Runs" sheetId="2" r:id="R0050cb5734004c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Outcomes" sheetId="3" r:id="Rbd34d2c65ec84487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sweep Runs" sheetId="4" r:id="Rfd55c807e1f64c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Runs" sheetId="5" r:id="R5fef01b4fb294ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Outcomes" sheetId="6" r:id="R759d8ba4148941c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" r:id="R78b7baacc6a643b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -666,13 +666,13 @@
         <x:v>Base</x:v>
       </x:c>
       <x:c r="C12" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D12" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E12" s="34" t="n">
-        <x:v>0.23529411764705882</x:v>
+        <x:v>0.35294117647058826</x:v>
       </x:c>
       <x:c r="F12" s="33" t="n">
         <x:v>0</x:v>
@@ -701,16 +701,16 @@
         <x:v>Qwen-HRM</x:v>
       </x:c>
       <x:c r="C13" s="33" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D13" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E13" s="34" t="n">
-        <x:v>0.29411764705882354</x:v>
+        <x:v>0.35294117647058826</x:v>
       </x:c>
       <x:c r="F13" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="35" t="n">
         <x:v>27.241536667996115</x:v>
@@ -736,20 +736,20 @@
         <x:v>HRM-Text</x:v>
       </x:c>
       <x:c r="C14" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D14" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E14" s="34" t="n">
-        <x:v>0.17647058823529413</x:v>
+        <x:v>0.9411764705882353</x:v>
       </x:c>
       <x:c r="F14" s="33" t="str"/>
       <x:c r="G14" s="35" t="n">
-        <x:v>39.10392216801483</x:v>
+        <x:v>104.68802758599998</x:v>
       </x:c>
       <x:c r="H14" s="35" t="n">
-        <x:v>2.3002307157655784</x:v>
+        <x:v>6.158119269764704</x:v>
       </x:c>
       <x:c r="I14" s="31"/>
       <x:c r="J14" s="31"/>
@@ -769,20 +769,20 @@
         <x:v>HRM-Text</x:v>
       </x:c>
       <x:c r="C15" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D15" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E15" s="34" t="n">
-        <x:v>0.058823529411764705</x:v>
+        <x:v>0.9411764705882353</x:v>
       </x:c>
       <x:c r="F15" s="33" t="str"/>
       <x:c r="G15" s="35" t="n">
-        <x:v>84.48929779399987</x:v>
+        <x:v>338.2124144539998</x:v>
       </x:c>
       <x:c r="H15" s="35" t="n">
-        <x:v>4.969958693764698</x:v>
+        <x:v>19.894847909058814</x:v>
       </x:c>
       <x:c r="I15" s="31"/>
       <x:c r="J15" s="31"/>
@@ -33854,8 +33854,8 @@
     <x:col min="5" max="5" width="10.430000305175781" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.430000305175781" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10.430000305175781" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="37.90999984741211" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="23.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="141.47000122070312" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="31.65999984741211" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -33977,13 +33977,13 @@
         <x:v>Base</x:v>
       </x:c>
       <x:c r="C4" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D4" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E4" s="34" t="n">
-        <x:v>0.23529411764705882</x:v>
+        <x:v>0.35294117647058826</x:v>
       </x:c>
       <x:c r="F4" s="35" t="n">
         <x:v>11.462043749994336</x:v>
@@ -33992,7 +33992,7 @@
         <x:v>0.6742378676467257</x:v>
       </x:c>
       <x:c r="H4" s="33" t="str">
-        <x:v>sequence, reverse_discount, average, coins</x:v>
+        <x:v>boxes, probability, sequence, reverse_discount, average, coins</x:v>
       </x:c>
       <x:c r="I4" s="33" t="str">
         <x:v>exact_qwen3_1_7b_base.csv</x:v>
@@ -34014,13 +34014,13 @@
         <x:v>Qwen-HRM</x:v>
       </x:c>
       <x:c r="C5" s="33" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D5" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E5" s="34" t="n">
-        <x:v>0.29411764705882354</x:v>
+        <x:v>0.35294117647058826</x:v>
       </x:c>
       <x:c r="F5" s="35" t="n">
         <x:v>27.241536667996115</x:v>
@@ -34029,7 +34029,7 @@
         <x:v>1.6024433334115362</x:v>
       </x:c>
       <x:c r="H5" s="33" t="str">
-        <x:v>markup, probability, sequence, rectangle, coins</x:v>
+        <x:v>markup, boxes, probability, sequence, rectangle, coins</x:v>
       </x:c>
       <x:c r="I5" s="33" t="str">
         <x:v>exact_qwen3_1_7b_hrm.csv</x:v>
@@ -34051,25 +34051,25 @@
         <x:v>HRM-Text</x:v>
       </x:c>
       <x:c r="C6" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D6" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>0.17647058823529413</x:v>
+        <x:v>0.9411764705882353</x:v>
       </x:c>
       <x:c r="F6" s="35" t="n">
-        <x:v>39.10392216801483</x:v>
+        <x:v>104.68802758599998</x:v>
       </x:c>
       <x:c r="G6" s="35" t="n">
-        <x:v>2.3002307157655784</x:v>
+        <x:v>6.158119269764704</x:v>
       </x:c>
       <x:c r="H6" s="33" t="str">
-        <x:v>sequence, average, modular_small</x:v>
+        <x:v>algebra, markup, boxes, inclusion, work_rate, probability, sequence, linear_word, reverse_discount, multiples, rectangle, average, combinations, coins, modular_small, syllogism</x:v>
       </x:c>
       <x:c r="I6" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="J6" s="31"/>
       <x:c r="K6" s="31"/>
@@ -34088,25 +34088,25 @@
         <x:v>HRM-Text</x:v>
       </x:c>
       <x:c r="C7" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D7" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="E7" s="34" t="n">
-        <x:v>0.058823529411764705</x:v>
+        <x:v>0.9411764705882353</x:v>
       </x:c>
       <x:c r="F7" s="35" t="n">
-        <x:v>84.48929779399987</x:v>
+        <x:v>338.2124144539998</x:v>
       </x:c>
       <x:c r="G7" s="35" t="n">
-        <x:v>4.969958693764698</x:v>
+        <x:v>19.894847909058814</x:v>
       </x:c>
       <x:c r="H7" s="33" t="str">
-        <x:v>syllogism</x:v>
+        <x:v>algebra, markup, boxes, inclusion, modular, work_rate, probability, sequence, linear_word, reverse_discount, multiples, rectangle, average, combinations, coins, syllogism</x:v>
       </x:c>
       <x:c r="I7" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="J7" s="31"/>
       <x:c r="K7" s="31"/>
@@ -39700,7 +39700,7 @@
     <x:col min="5" max="5" width="255" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10.430000305175781" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="23.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="31.65999984741211" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -39786,9 +39786,7 @@
       <x:c r="D3" s="33" t="str">
         <x:v>96|$96</x:v>
       </x:c>
-      <x:c r="E3" s="33" t="str">
-        <x:v>Hmm, let's break it down step by step. Let me think. When something is marked up by 25%, that means the original price is reduced by 25% of the original price. Wait, no, actually, when you mark up something, you're increasing its</x:v>
-      </x:c>
+      <x:c r="E3" s="33" t="str"/>
       <x:c r="F3" s="33" t="str">
         <x:v>False</x:v>
       </x:c>
@@ -40555,7 +40553,7 @@
         <x:v>1/9</x:v>
       </x:c>
       <x:c r="E25" s="33" t="str">
-        <x:v>'- 4: 4 + 4 = 8</x:v>
+        <x:v>\text{answer}</x:v>
       </x:c>
       <x:c r="F25" s="33" t="str">
         <x:v>False</x:v>
@@ -41013,7 +41011,7 @@
         <x:v>To determine which box to open, we need to figure out the correct labels based on the information given. Since all the labels are wrong, we can use the fact that the Mixed box is the only one that could have both apples and oranges. If we take one fruit from the Mixed box, we can determine if it's apples or oranges. If it's apples, then the Mixed box is actually apples, but since all labels are wrong, the Mixed box can't be correct. If it's oranges, then the Mixed box is actually oranges, but since all labels are wrong, the Mixed box can't be correct. Therefore,</x:v>
       </x:c>
       <x:c r="F38" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G38" s="35" t="n">
         <x:v>0.6743095830024686</x:v>
@@ -41153,7 +41151,7 @@
         <x:v>\boxed{\dfrac{1}{9}}.</x:v>
       </x:c>
       <x:c r="F42" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G42" s="35" t="n">
         <x:v>0.667745416998514</x:v>
@@ -41608,7 +41606,7 @@
         <x:v>Now, the "Mixed" box must have either apples</x:v>
       </x:c>
       <x:c r="F55" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G55" s="35" t="n">
         <x:v>1.6641501670019352</x:v>
@@ -42130,16 +42128,16 @@
         <x:v>12.5|25/2</x:v>
       </x:c>
       <x:c r="E70" s="33" t="str">
-        <x:v>Step 4: Add 21 to both sides of the equation to isolate the</x:v>
+        <x:v>\dfrac{25}{2}</x:v>
       </x:c>
       <x:c r="F70" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G70" s="35" t="n">
-        <x:v>2.7778973340027733</x:v>
+        <x:v>7.580443959000007</x:v>
       </x:c>
       <x:c r="H70" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I70" s="31"/>
       <x:c r="J70" s="31"/>
@@ -42165,16 +42163,16 @@
         <x:v>96|$96</x:v>
       </x:c>
       <x:c r="E71" s="33" t="str">
-        <x:v>4. Calculate the product of 1.25 and 0.8</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F71" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G71" s="35" t="n">
-        <x:v>2.734651083999779</x:v>
+        <x:v>6.407860625000012</x:v>
       </x:c>
       <x:c r="H71" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I71" s="31"/>
       <x:c r="J71" s="31"/>
@@ -42200,16 +42198,16 @@
         <x:v>mixed|Mixed</x:v>
       </x:c>
       <x:c r="E72" s="33" t="str">
-        <x:v>your answer**</x:v>
+        <x:v>Mixed</x:v>
       </x:c>
       <x:c r="F72" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G72" s="35" t="n">
-        <x:v>2.5394804999996268</x:v>
+        <x:v>6.2715228750000165</x:v>
       </x:c>
       <x:c r="H72" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I72" s="31"/>
       <x:c r="J72" s="31"/>
@@ -42235,16 +42233,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E73" s="33" t="str">
-        <x:v>The largest multiple of 5 less than or equal to 200 is 200. So, the number of</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F73" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G73" s="35" t="n">
-        <x:v>2.6089392920002865</x:v>
+        <x:v>4.775222624999998</x:v>
       </x:c>
       <x:c r="H73" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I73" s="31"/>
       <x:c r="J73" s="31"/>
@@ -42270,16 +42268,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E74" s="33" t="str">
-        <x:v>7^6 ≡ 7 * 11 ≡ 7</x:v>
+        <x:v>'- \(7^8 \equiv 9^2</x:v>
       </x:c>
       <x:c r="F74" s="33" t="str">
         <x:v>False</x:v>
       </x:c>
       <x:c r="G74" s="35" t="n">
-        <x:v>2.560868417000165</x:v>
+        <x:v>14.03727679100001</x:v>
       </x:c>
       <x:c r="H74" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I74" s="31"/>
       <x:c r="J74" s="31"/>
@@ -42305,16 +42303,16 @@
         <x:v>3.75|15/4</x:v>
       </x:c>
       <x:c r="E75" s="33" t="str">
-        <x:v>\frac{1}{6} = \frac{5}{30} \quad \text{and} \</x:v>
+        <x:v>\dfrac{15}{4}</x:v>
       </x:c>
       <x:c r="F75" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G75" s="35" t="n">
-        <x:v>2.554322083000443</x:v>
+        <x:v>6.176148500000011</x:v>
       </x:c>
       <x:c r="H75" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I75" s="31"/>
       <x:c r="J75" s="31"/>
@@ -42340,16 +42338,16 @@
         <x:v>1/9</x:v>
       </x:c>
       <x:c r="E76" s="33" t="str">
-        <x:v>your answer</x:v>
+        <x:v>\dfrac{1}{9}</x:v>
       </x:c>
       <x:c r="F76" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G76" s="35" t="n">
-        <x:v>1.3759969169987016</x:v>
+        <x:v>4.10938950000002</x:v>
       </x:c>
       <x:c r="H76" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I76" s="31"/>
       <x:c r="J76" s="31"/>
@@ -42381,10 +42379,10 @@
         <x:v>True</x:v>
       </x:c>
       <x:c r="G77" s="35" t="n">
-        <x:v>2.2476258749993576</x:v>
+        <x:v>8.457965874999957</x:v>
       </x:c>
       <x:c r="H77" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I77" s="31"/>
       <x:c r="J77" s="31"/>
@@ -42410,16 +42408,16 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E78" s="33" t="str">
-        <x:v>2x &amp;= 31 - 9 \\</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F78" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G78" s="35" t="n">
-        <x:v>2.5328067080008623</x:v>
+        <x:v>4.77963704199999</x:v>
       </x:c>
       <x:c r="H78" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I78" s="31"/>
       <x:c r="J78" s="31"/>
@@ -42445,16 +42443,16 @@
         <x:v>80|$80</x:v>
       </x:c>
       <x:c r="E79" s="33" t="str">
-        <x:v>P = \frac{</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F79" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G79" s="35" t="n">
-        <x:v>2.9531720420018246</x:v>
+        <x:v>4.465110458999959</x:v>
       </x:c>
       <x:c r="H79" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I79" s="31"/>
       <x:c r="J79" s="31"/>
@@ -42480,16 +42478,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E80" s="33" t="str">
-        <x:v>The largest integer less than 100 that is divisible by</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F80" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G80" s="35" t="n">
-        <x:v>2.88598975000059</x:v>
+        <x:v>4.0312850840000465</x:v>
       </x:c>
       <x:c r="H80" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I80" s="31"/>
       <x:c r="J80" s="31"/>
@@ -42515,16 +42513,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E81" s="33" t="str">
-        <x:v>3. **Solve</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F81" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G81" s="35" t="n">
-        <x:v>2.7802965410010074</x:v>
+        <x:v>4.098184124999989</x:v>
       </x:c>
       <x:c r="H81" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I81" s="31"/>
       <x:c r="J81" s="31"/>
@@ -42556,10 +42554,10 @@
         <x:v>True</x:v>
       </x:c>
       <x:c r="G82" s="35" t="n">
-        <x:v>2.5419051670032786</x:v>
+        <x:v>3.955258875000027</x:v>
       </x:c>
       <x:c r="H82" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I82" s="31"/>
       <x:c r="J82" s="31"/>
@@ -42585,16 +42583,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E83" s="33" t="str">
-        <x:v>= (6 × 5 × 4 × 3 × 2 × 1) / ((2 × 1)(4 × 3</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F83" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G83" s="35" t="n">
-        <x:v>2.8596924170014972</x:v>
+        <x:v>6.499252583999976</x:v>
       </x:c>
       <x:c r="H83" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I83" s="31"/>
       <x:c r="J83" s="31"/>
@@ -42620,16 +42618,16 @@
         <x:v>3/8</x:v>
       </x:c>
       <x:c r="E84" s="33" t="str">
-        <x:v>$\boxed{\frac{3}{8}}$</x:v>
+        <x:v>\dfrac{3}{8}</x:v>
       </x:c>
       <x:c r="F84" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G84" s="35" t="n">
-        <x:v>1.3579884579994541</x:v>
+        <x:v>2.2782300830000395</x:v>
       </x:c>
       <x:c r="H84" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I84" s="31"/>
       <x:c r="J84" s="31"/>
@@ -42661,10 +42659,10 @@
         <x:v>True</x:v>
       </x:c>
       <x:c r="G85" s="35" t="n">
-        <x:v>1.2371588330024679</x:v>
+        <x:v>12.253404416999956</x:v>
       </x:c>
       <x:c r="H85" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I85" s="31"/>
       <x:c r="J85" s="31"/>
@@ -42690,16 +42688,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="E86" s="33" t="str">
-        <x:v>your answer</x:v>
+        <x:v>Yes, all bloops must be lazzies.</x:v>
       </x:c>
       <x:c r="F86" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G86" s="35" t="n">
-        <x:v>0.5551307500027178</x:v>
+        <x:v>4.511834166999961</x:v>
       </x:c>
       <x:c r="H86" s="33" t="str">
-        <x:v>exact_hrm_text_1b_4bit.csv</x:v>
+        <x:v>exact_hrm_text_1b_4bit_corrected.csv</x:v>
       </x:c>
       <x:c r="I86" s="31"/>
       <x:c r="J86" s="31"/>
@@ -42725,16 +42723,16 @@
         <x:v>12.5|25/2</x:v>
       </x:c>
       <x:c r="E87" s="33" t="str">
-        <x:v>Step 4: Add 21 to both sides of the equation to isolate</x:v>
+        <x:v>\dfrac{25}{2}</x:v>
       </x:c>
       <x:c r="F87" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G87" s="35" t="n">
-        <x:v>5.188138792000245</x:v>
+        <x:v>16.656210082999962</x:v>
       </x:c>
       <x:c r="H87" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I87" s="31"/>
       <x:c r="J87" s="31"/>
@@ -42760,16 +42758,16 @@
         <x:v>96|$96</x:v>
       </x:c>
       <x:c r="E88" s="33" t="str">
-        <x:v>4. Calculate the product of 1.25 and 0.8</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F88" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G88" s="35" t="n">
-        <x:v>5.103107375001855</x:v>
+        <x:v>12.64156225000005</x:v>
       </x:c>
       <x:c r="H88" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I88" s="31"/>
       <x:c r="J88" s="31"/>
@@ -42795,16 +42793,16 @@
         <x:v>mixed|Mixed</x:v>
       </x:c>
       <x:c r="E89" s="33" t="str">
-        <x:v>your answer**</x:v>
+        <x:v>**Final Answer**: The fruit is drawn from the **Mixed** box.</x:v>
       </x:c>
       <x:c r="F89" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G89" s="35" t="n">
-        <x:v>4.371220457996969</x:v>
+        <x:v>19.97141316599999</x:v>
       </x:c>
       <x:c r="H89" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I89" s="31"/>
       <x:c r="J89" s="31"/>
@@ -42830,16 +42828,16 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E90" s="33" t="str">
-        <x:v>The largest integer less than or equal to 200 that is divisible by 5 is 200. So,</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F90" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G90" s="35" t="n">
-        <x:v>5.096478874998866</x:v>
+        <x:v>12.902716834000046</x:v>
       </x:c>
       <x:c r="H90" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I90" s="31"/>
       <x:c r="J90" s="31"/>
@@ -42865,16 +42863,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E91" s="33" t="str">
-        <x:v>\[ 7^{103} = 7^{12 \times</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F91" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G91" s="35" t="n">
-        <x:v>5.095068083999649</x:v>
+        <x:v>50.31506079099995</x:v>
       </x:c>
       <x:c r="H91" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I91" s="31"/>
       <x:c r="J91" s="31"/>
@@ -42900,16 +42898,16 @@
         <x:v>3.75|15/4</x:v>
       </x:c>
       <x:c r="E92" s="33" t="str">
-        <x:v>\frac{1}{6} = \frac{5}{30} \quad \text{and} \quad \frac{1}{10} = \frac{3}{</x:v>
+        <x:v>3.75</x:v>
       </x:c>
       <x:c r="F92" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G92" s="35" t="n">
-        <x:v>5.09630420800022</x:v>
+        <x:v>33.462693083999966</x:v>
       </x:c>
       <x:c r="H92" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I92" s="31"/>
       <x:c r="J92" s="31"/>
@@ -42935,16 +42933,16 @@
         <x:v>1/9</x:v>
       </x:c>
       <x:c r="E93" s="33" t="str">
-        <x:v>your answer</x:v>
+        <x:v>\dfrac{1}{9}</x:v>
       </x:c>
       <x:c r="F93" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G93" s="35" t="n">
-        <x:v>2.531712209001853</x:v>
+        <x:v>7.085368707999919</x:v>
       </x:c>
       <x:c r="H93" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I93" s="31"/>
       <x:c r="J93" s="31"/>
@@ -42970,16 +42968,16 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="E94" s="33" t="str">
-        <x:v>So, a_4 = \</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F94" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G94" s="35" t="n">
-        <x:v>5.103402249998908</x:v>
+        <x:v>15.824353458000019</x:v>
       </x:c>
       <x:c r="H94" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I94" s="31"/>
       <x:c r="J94" s="31"/>
@@ -43005,16 +43003,16 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E95" s="33" t="str">
-        <x:v>2x &amp;= 22 \\</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F95" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G95" s="35" t="n">
-        <x:v>5.092639833997964</x:v>
+        <x:v>8.149854707999907</x:v>
       </x:c>
       <x:c r="H95" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I95" s="31"/>
       <x:c r="J95" s="31"/>
@@ -43040,16 +43038,16 @@
         <x:v>80|$80</x:v>
       </x:c>
       <x:c r="E96" s="33" t="str">
-        <x:v>Verification: A 10% discount on $80 is $8, so the discounted price is $80 - $8 = $72, which matches</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F96" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G96" s="35" t="n">
-        <x:v>5.0926331669979845</x:v>
+        <x:v>6.157211500000017</x:v>
       </x:c>
       <x:c r="H96" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I96" s="31"/>
       <x:c r="J96" s="31"/>
@@ -43075,16 +43073,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E97" s="33" t="str">
-        <x:v>The largest integer less than 100 that is divisible by</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F97" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G97" s="35" t="n">
-        <x:v>5.080499875002715</x:v>
+        <x:v>21.503388040999994</x:v>
       </x:c>
       <x:c r="H97" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I97" s="31"/>
       <x:c r="J97" s="31"/>
@@ -43110,16 +43108,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E98" s="33" t="str">
-        <x:v>3. **Solve</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F98" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G98" s="35" t="n">
-        <x:v>5.522503542000777</x:v>
+        <x:v>7.560139790999983</x:v>
       </x:c>
       <x:c r="H98" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I98" s="31"/>
       <x:c r="J98" s="31"/>
@@ -43145,16 +43143,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E99" s="33" t="str">
-        <x:v>Thus</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F99" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G99" s="35" t="n">
-        <x:v>5.390843000001041</x:v>
+        <x:v>8.231041165999955</x:v>
       </x:c>
       <x:c r="H99" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I99" s="31"/>
       <x:c r="J99" s="31"/>
@@ -43180,16 +43178,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E100" s="33" t="str">
-        <x:v>\[ 6! = 6 \times 5 \times</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F100" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G100" s="35" t="n">
-        <x:v>5.357839625001361</x:v>
+        <x:v>30.73365029099989</x:v>
       </x:c>
       <x:c r="H100" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I100" s="31"/>
       <x:c r="J100" s="31"/>
@@ -43215,16 +43213,16 @@
         <x:v>3/8</x:v>
       </x:c>
       <x:c r="E101" s="33" t="str">
-        <x:v>There are 3 favorable outcomes. The probability is calculated by dividing the number of favorable outcomes by t</x:v>
+        <x:v>\dfrac{3}{8}</x:v>
       </x:c>
       <x:c r="F101" s="33" t="str">
-        <x:v>False</x:v>
+        <x:v>True</x:v>
       </x:c>
       <x:c r="G101" s="35" t="n">
-        <x:v>5.398683916999289</x:v>
+        <x:v>11.049620875000073</x:v>
       </x:c>
       <x:c r="H101" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I101" s="31"/>
       <x:c r="J101" s="31"/>
@@ -43250,16 +43248,16 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E102" s="33" t="str">
-        <x:v>\[ \</x:v>
+        <x:v>All methods confirm that the remainder when</x:v>
       </x:c>
       <x:c r="F102" s="33" t="str">
         <x:v>False</x:v>
       </x:c>
       <x:c r="G102" s="35" t="n">
-        <x:v>5.481146750000335</x:v>
+        <x:v>67.06586500000003</x:v>
       </x:c>
       <x:c r="H102" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I102" s="31"/>
       <x:c r="J102" s="31"/>
@@ -43285,16 +43283,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="E103" s="33" t="str">
-        <x:v>Final answer: yes</x:v>
+        <x:v>Yes, all bloops must be lazzies.</x:v>
       </x:c>
       <x:c r="F103" s="33" t="str">
         <x:v>True</x:v>
       </x:c>
       <x:c r="G103" s="35" t="n">
-        <x:v>4.487075832999835</x:v>
+        <x:v>8.902264708000075</x:v>
       </x:c>
       <x:c r="H103" s="33" t="str">
-        <x:v>exact_hrm_text_1b_bf16.csv</x:v>
+        <x:v>exact_hrm_text_1b_bf16_corrected.csv</x:v>
       </x:c>
       <x:c r="I103" s="31"/>
       <x:c r="J103" s="31"/>
@@ -47059,7 +47057,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18.040000915527344" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="125.5199966430664" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="150.17999267578125" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -47159,7 +47157,7 @@
         <x:v>Exact-answer probe</x:v>
       </x:c>
       <x:c r="B5" s="41" t="str">
-        <x:v>Added a stricter generative probe with exact extraction. Qwen3-0.6B moves from 1/17 base to 2/17 HRM; Qwen3-1.7B moves from 4/17 base to 5/17 HRM.</x:v>
+        <x:v>Added a stricter generative probe with exact extraction. Qwen3-0.6B moves from 1/17 base to 2/17 HRM; Qwen3-1.7B is 6/17 for both base and HRM after corrected text-answer scoring.</x:v>
       </x:c>
       <x:c r="C5" s="31"/>
       <x:c r="D5" s="31"/>
@@ -47182,7 +47180,7 @@
         <x:v>HRM-Text comparison</x:v>
       </x:c>
       <x:c r="B6" s="41" t="str">
-        <x:v>Local HRM-Text-1B scored 3/17 for 4-bit and 1/17 for BF16 on this exact prompt set; treat this as prompt-sensitive, not a definitive model ranking.</x:v>
+        <x:v>The original HRM-Text exact run used the wrong final-answer prompt/extraction and too small a token cap. Corrected boxed-prompt runs score 16/17 for both 4-bit and BF16.</x:v>
       </x:c>
       <x:c r="C6" s="31"/>
       <x:c r="D6" s="31"/>

</xml_diff>

<commit_message>
Track Qwen 0.6B ARC probe results
</commit_message>
<xml_diff>
--- a/outputs/qwen_hrm_metrics/qwen_hrm_conversion_metrics.xlsx
+++ b/outputs/qwen_hrm_metrics/qwen_hrm_conversion_metrics.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5ea8e0be52154fe2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Runs" sheetId="2" r:id="R4e0962bfe8f64468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Outcomes" sheetId="3" r:id="R22ea8a6a15f848f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sweep Runs" sheetId="4" r:id="Rec4894bd3c114b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Runs" sheetId="5" r:id="R32a330b52c304f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Outcomes" sheetId="6" r:id="R79e54b233ded419a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rerank Runs" sheetId="7" r:id="R8c7f475fd7af43c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARC Runs" sheetId="8" r:id="Rc1acf40dc848486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="Rac6afbdc9add40da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R71cce2d008924dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Runs" sheetId="2" r:id="Re83cb8e2212a45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Outcomes" sheetId="3" r:id="R762bf780269046cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sweep Runs" sheetId="4" r:id="R1d880d7f8350426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Runs" sheetId="5" r:id="Ra792174f4d03435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exact Outcomes" sheetId="6" r:id="R6bdffbf681d743a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rerank Runs" sheetId="7" r:id="R20db5caa25844681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARC Runs" sheetId="8" r:id="Rca98ba1ba11f44b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" r:id="R5b87ed333cd746b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56972,7 +56972,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="33" t="str">
-        <x:v>Qwen3-1.7B-4bit</x:v>
+        <x:v>Qwen3-0.6B-4bit</x:v>
       </x:c>
       <x:c r="B2" s="33" t="str">
         <x:v>validation</x:v>
@@ -56990,19 +56990,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="33" t="n">
-        <x:v>37</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H2" s="33" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="I2" s="34" t="n">
-        <x:v>0.74</x:v>
+        <x:v>0.42</x:v>
       </x:c>
       <x:c r="J2" s="35" t="n">
-        <x:v>7.229978584000037</x:v>
+        <x:v>3.20136787499996</x:v>
       </x:c>
       <x:c r="K2" s="33" t="str">
-        <x:v>arc_qwen3_1_7b_base_validation50.csv</x:v>
+        <x:v>arc_qwen3_0_6b_base_validation50.csv</x:v>
       </x:c>
       <x:c r="L2" s="31"/>
       <x:c r="M2" s="31"/>
@@ -57013,7 +57013,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33" t="str">
-        <x:v>Qwen3-1.7B-4bit</x:v>
+        <x:v>Qwen3-0.6B-4bit</x:v>
       </x:c>
       <x:c r="B3" s="33" t="str">
         <x:v>validation</x:v>
@@ -57031,19 +57031,19 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="G3" s="33" t="n">
-        <x:v>35</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H3" s="33" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="I3" s="34" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.42</x:v>
       </x:c>
       <x:c r="J3" s="35" t="n">
-        <x:v>20.041542333000052</x:v>
+        <x:v>8.204612542000177</x:v>
       </x:c>
       <x:c r="K3" s="33" t="str">
-        <x:v>arc_qwen3_1_7b_hrm_validation50.csv</x:v>
+        <x:v>arc_qwen3_0_6b_hrm_validation50.csv</x:v>
       </x:c>
       <x:c r="L3" s="31"/>
       <x:c r="M3" s="31"/>
@@ -57054,7 +57054,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="33" t="str">
-        <x:v>Qwen3-1.7B-4bit</x:v>
+        <x:v>Qwen3-0.6B-4bit</x:v>
       </x:c>
       <x:c r="B4" s="33" t="str">
         <x:v>validation</x:v>
@@ -57072,19 +57072,19 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="G4" s="33" t="n">
-        <x:v>37</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H4" s="33" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="I4" s="34" t="n">
-        <x:v>0.74</x:v>
+        <x:v>0.42</x:v>
       </x:c>
       <x:c r="J4" s="35" t="n">
-        <x:v>20.54996462500003</x:v>
+        <x:v>8.522171374999743</x:v>
       </x:c>
       <x:c r="K4" s="33" t="str">
-        <x:v>arc_qwen3_1_7b_hrm_agreement_validation50.csv</x:v>
+        <x:v>arc_qwen3_0_6b_hrm_agreement_validation50.csv</x:v>
       </x:c>
       <x:c r="L4" s="31"/>
       <x:c r="M4" s="31"/>
@@ -57094,17 +57094,39 @@
       <x:c r="Q4" s="31"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="31"/>
-      <x:c r="B5" s="31"/>
-      <x:c r="C5" s="31"/>
-      <x:c r="D5" s="31"/>
-      <x:c r="E5" s="31"/>
-      <x:c r="F5" s="31"/>
-      <x:c r="G5" s="31"/>
-      <x:c r="H5" s="31"/>
-      <x:c r="I5" s="36"/>
-      <x:c r="J5" s="37"/>
-      <x:c r="K5" s="31"/>
+      <x:c r="A5" s="33" t="str">
+        <x:v>Qwen3-1.7B-4bit</x:v>
+      </x:c>
+      <x:c r="B5" s="33" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="C5" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D5" s="33" t="str">
+        <x:v>base</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="str">
+        <x:v>blend</x:v>
+      </x:c>
+      <x:c r="F5" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="33" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="H5" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I5" s="34" t="n">
+        <x:v>0.74</x:v>
+      </x:c>
+      <x:c r="J5" s="35" t="n">
+        <x:v>7.229978584000037</x:v>
+      </x:c>
+      <x:c r="K5" s="33" t="str">
+        <x:v>arc_qwen3_1_7b_base_validation50.csv</x:v>
+      </x:c>
       <x:c r="L5" s="31"/>
       <x:c r="M5" s="31"/>
       <x:c r="N5" s="31"/>
@@ -57113,17 +57135,39 @@
       <x:c r="Q5" s="31"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="31"/>
-      <x:c r="B6" s="31"/>
-      <x:c r="C6" s="31"/>
-      <x:c r="D6" s="31"/>
-      <x:c r="E6" s="31"/>
-      <x:c r="F6" s="31"/>
-      <x:c r="G6" s="31"/>
-      <x:c r="H6" s="31"/>
-      <x:c r="I6" s="36"/>
-      <x:c r="J6" s="37"/>
-      <x:c r="K6" s="31"/>
+      <x:c r="A6" s="33" t="str">
+        <x:v>Qwen3-1.7B-4bit</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="C6" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="str">
+        <x:v>hrm</x:v>
+      </x:c>
+      <x:c r="E6" s="33" t="str">
+        <x:v>blend</x:v>
+      </x:c>
+      <x:c r="F6" s="33" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="G6" s="33" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H6" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I6" s="34" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="J6" s="35" t="n">
+        <x:v>20.041542333000052</x:v>
+      </x:c>
+      <x:c r="K6" s="33" t="str">
+        <x:v>arc_qwen3_1_7b_hrm_validation50.csv</x:v>
+      </x:c>
       <x:c r="L6" s="31"/>
       <x:c r="M6" s="31"/>
       <x:c r="N6" s="31"/>
@@ -57132,17 +57176,39 @@
       <x:c r="Q6" s="31"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="31"/>
-      <x:c r="B7" s="31"/>
-      <x:c r="C7" s="31"/>
-      <x:c r="D7" s="31"/>
-      <x:c r="E7" s="31"/>
-      <x:c r="F7" s="31"/>
-      <x:c r="G7" s="31"/>
-      <x:c r="H7" s="31"/>
-      <x:c r="I7" s="36"/>
-      <x:c r="J7" s="37"/>
-      <x:c r="K7" s="31"/>
+      <x:c r="A7" s="33" t="str">
+        <x:v>Qwen3-1.7B-4bit</x:v>
+      </x:c>
+      <x:c r="B7" s="33" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="C7" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D7" s="33" t="str">
+        <x:v>hrm</x:v>
+      </x:c>
+      <x:c r="E7" s="33" t="str">
+        <x:v>agreement_blend</x:v>
+      </x:c>
+      <x:c r="F7" s="33" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="G7" s="33" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="H7" s="33" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I7" s="34" t="n">
+        <x:v>0.74</x:v>
+      </x:c>
+      <x:c r="J7" s="35" t="n">
+        <x:v>20.54996462500003</x:v>
+      </x:c>
+      <x:c r="K7" s="33" t="str">
+        <x:v>arc_qwen3_1_7b_hrm_agreement_validation50.csv</x:v>
+      </x:c>
       <x:c r="L7" s="31"/>
       <x:c r="M7" s="31"/>
       <x:c r="N7" s="31"/>
@@ -62727,7 +62793,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18.040000915527344" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="150.6699981689453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="156.1999969482422" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -62919,7 +62985,7 @@
         <x:v>ARC-Challenge slice</x:v>
       </x:c>
       <x:c r="B9" s="41" t="str">
-        <x:v>On ARC-Challenge validation[:50], Qwen3-1.7B base scores 37/50, fixed HRM blend scores 35/50, and agreement_blend recovers 37/50.</x:v>
+        <x:v>On ARC-Challenge validation[:50], Qwen3-0.6B is flat at 21/50 for base, fixed blend, and agreement_blend; Qwen3-1.7B base is 37/50, fixed blend is 35/50, and agreement_blend recovers 37/50.</x:v>
       </x:c>
       <x:c r="C9" s="31"/>
       <x:c r="D9" s="31"/>

</xml_diff>